<commit_message>
Replaced +/- SD with central 2/3ds.
</commit_message>
<xml_diff>
--- a/data/ref_pop-2026-03-20.xlsx
+++ b/data/ref_pop-2026-03-20.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeanettemelin/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hakanjo\ProtonDrive\My files\forskningssektionen\projects-current\jeanette_melin-shiny\elderly_wellbeing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2374195A-722F-164A-A5C9-2D8FD84F926E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E16303-8EAC-46CA-AE31-0B983AB773DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24280" yWindow="7100" windowWidth="28240" windowHeight="17240" xr2:uid="{37809B56-4A83-7B42-93FB-B3F3B8C0AE69}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{37809B56-4A83-7B42-93FB-B3F3B8C0AE69}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
   <si>
     <t>Medelvärde</t>
   </si>
@@ -90,6 +90,12 @@
   </si>
   <si>
     <t> 46-71</t>
+  </si>
+  <si>
+    <t>q_1_6</t>
+  </si>
+  <si>
+    <t>q_5_6</t>
   </si>
 </sst>
 </file>
@@ -145,10 +151,12 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -169,7 +177,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -485,149 +493,197 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F638BF61-FA25-0549-BAC0-EA20ABD1A0F5}">
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="10.83203125" style="3"/>
+    <col min="1" max="1" width="18.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="10.875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="F1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>60</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
         <v>14</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="F2" s="4">
+        <v>48</v>
+      </c>
+      <c r="G2" s="3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>59</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>14</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="F3" s="4">
+        <v>46</v>
+      </c>
+      <c r="G3" s="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>61</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>13</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="F4" s="4">
+        <v>48</v>
+      </c>
+      <c r="G4" s="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>62</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>14</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="F5" s="4">
+        <v>48</v>
+      </c>
+      <c r="G5" s="4">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>60</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>13</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="F6" s="4">
+        <v>46</v>
+      </c>
+      <c r="G6" s="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>61</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="3">
         <v>14</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+      <c r="F7" s="4">
+        <v>48</v>
+      </c>
+      <c r="G7" s="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>59</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="3">
         <v>13</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
+      <c r="F8" s="4">
+        <v>46</v>
+      </c>
+      <c r="G8" s="4">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A9" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Minor tweaks to the plots and tables.
</commit_message>
<xml_diff>
--- a/data/ref_pop-2026-03-20.xlsx
+++ b/data/ref_pop-2026-03-20.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hakanjo\ProtonDrive\My files\forskningssektionen\projects-current\jeanette_melin-shiny\elderly_wellbeing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53E16303-8EAC-46CA-AE31-0B983AB773DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9CD940-D41C-43C4-9EBC-07E02A37CB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{37809B56-4A83-7B42-93FB-B3F3B8C0AE69}"/>
   </bookViews>
@@ -50,45 +50,24 @@
     <t>2/3 range</t>
   </si>
   <si>
-    <t>Totalt</t>
-  </si>
-  <si>
     <t> 62</t>
   </si>
   <si>
     <t>  48-73 </t>
   </si>
   <si>
-    <t>Män</t>
-  </si>
-  <si>
     <t> 60</t>
   </si>
   <si>
     <t> 46-73</t>
   </si>
   <si>
-    <t>Kvinnor</t>
-  </si>
-  <si>
     <t> 48-73</t>
   </si>
   <si>
-    <t>79 år och yngre</t>
-  </si>
-  <si>
     <t> 48-76</t>
   </si>
   <si>
-    <t>80 år och äldre</t>
-  </si>
-  <si>
-    <t>Född i Sverige</t>
-  </si>
-  <si>
-    <t>Född utanför Sverige</t>
-  </si>
-  <si>
     <t> 46-71</t>
   </si>
   <si>
@@ -96,6 +75,27 @@
   </si>
   <si>
     <t>q_5_6</t>
+  </si>
+  <si>
+    <t>Totalt (ref.)</t>
+  </si>
+  <si>
+    <t>Män (ref.)</t>
+  </si>
+  <si>
+    <t>Kvinnor (ref.)</t>
+  </si>
+  <si>
+    <t>79 år och yngre (ref.)</t>
+  </si>
+  <si>
+    <t>80 år och äldre (ref.)</t>
+  </si>
+  <si>
+    <t>Född i Sverige (ref.)</t>
+  </si>
+  <si>
+    <t>Född utanför Sverige (ref.)</t>
   </si>
 </sst>
 </file>
@@ -515,15 +515,15 @@
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B2" s="3">
         <v>60</v>
@@ -532,10 +532,10 @@
         <v>14</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>6</v>
       </c>
       <c r="F2" s="4">
         <v>48</v>
@@ -546,7 +546,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B3" s="3">
         <v>59</v>
@@ -555,10 +555,10 @@
         <v>14</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F3" s="4">
         <v>46</v>
@@ -569,7 +569,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B4" s="3">
         <v>61</v>
@@ -578,10 +578,10 @@
         <v>13</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F4" s="4">
         <v>48</v>
@@ -592,7 +592,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B5" s="3">
         <v>62</v>
@@ -601,10 +601,10 @@
         <v>14</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F5" s="4">
         <v>48</v>
@@ -615,7 +615,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B6" s="3">
         <v>60</v>
@@ -624,10 +624,10 @@
         <v>13</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F6" s="4">
         <v>46</v>
@@ -638,7 +638,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B7" s="3">
         <v>61</v>
@@ -647,10 +647,10 @@
         <v>14</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F7" s="4">
         <v>48</v>
@@ -661,7 +661,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B8" s="3">
         <v>59</v>
@@ -670,10 +670,10 @@
         <v>13</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F8" s="4">
         <v>46</v>

</xml_diff>

<commit_message>
Removed medians and did some minor locale adjustments.
</commit_message>
<xml_diff>
--- a/data/ref_pop-2026-03-20.xlsx
+++ b/data/ref_pop-2026-03-20.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hakanjo\ProtonDrive\My files\forskningssektionen\projects-current\jeanette_melin-shiny\elderly_wellbeing\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hakanjo\ProtonDrive\My files\forskningssektionen\projects-current\jeanette_melin-shiny\share\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9CD940-D41C-43C4-9EBC-07E02A37CB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DB6ABB-8CB4-4B30-8BA9-AFD70C1A272C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{37809B56-4A83-7B42-93FB-B3F3B8C0AE69}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11835" xr2:uid="{37809B56-4A83-7B42-93FB-B3F3B8C0AE69}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>Medelvärde</t>
   </si>
@@ -50,59 +50,56 @@
     <t>2/3 range</t>
   </si>
   <si>
+    <t>Totalt</t>
+  </si>
+  <si>
     <t> 62</t>
   </si>
   <si>
     <t>  48-73 </t>
   </si>
   <si>
+    <t>Män</t>
+  </si>
+  <si>
     <t> 60</t>
   </si>
   <si>
     <t> 46-73</t>
   </si>
   <si>
+    <t>Kvinnor</t>
+  </si>
+  <si>
     <t> 48-73</t>
   </si>
   <si>
+    <t>79 år och yngre</t>
+  </si>
+  <si>
     <t> 48-76</t>
   </si>
   <si>
+    <t>80 år och äldre</t>
+  </si>
+  <si>
+    <t>Född i Sverige</t>
+  </si>
+  <si>
+    <t>Född utanför Sverige</t>
+  </si>
+  <si>
     <t> 46-71</t>
   </si>
   <si>
-    <t>q_1_6</t>
-  </si>
-  <si>
-    <t>q_5_6</t>
-  </si>
-  <si>
-    <t>Totalt (ref.)</t>
-  </si>
-  <si>
-    <t>Män (ref.)</t>
-  </si>
-  <si>
-    <t>Kvinnor (ref.)</t>
-  </si>
-  <si>
-    <t>79 år och yngre (ref.)</t>
-  </si>
-  <si>
-    <t>80 år och äldre (ref.)</t>
-  </si>
-  <si>
-    <t>Född i Sverige (ref.)</t>
-  </si>
-  <si>
-    <t>Född utanför Sverige (ref.)</t>
+    <t>N</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -128,6 +125,17 @@
       <name val="Calibri Light"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -137,7 +145,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -145,20 +153,47 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,197 +528,234 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F638BF61-FA25-0549-BAC0-EA20ABD1A0F5}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="10.875" style="2"/>
+    <col min="1" max="1" width="18.125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="10.875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="4">
+        <v>60</v>
+      </c>
+      <c r="C2" s="4">
+        <v>14</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="5">
+        <v>1187</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4">
+        <v>59</v>
+      </c>
+      <c r="C3" s="4">
+        <v>14</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="5">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="4">
+        <v>61</v>
+      </c>
+      <c r="C4" s="4">
+        <v>13</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="F4" s="5">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="B5" s="4">
+        <v>62</v>
+      </c>
+      <c r="C5" s="4">
+        <v>14</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="3">
+      <c r="F5" s="5">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="4">
         <v>60</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C6" s="4">
+        <v>13</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="5">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="4">
+        <v>61</v>
+      </c>
+      <c r="C7" s="4">
         <v>14</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="4">
-        <v>48</v>
-      </c>
-      <c r="G2" s="3">
+      <c r="E7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="5">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4">
+        <v>59</v>
+      </c>
+      <c r="C8" s="4">
+        <v>13</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="6">
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="3">
-        <v>59</v>
-      </c>
-      <c r="C3" s="3">
-        <v>14</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="4">
-        <v>46</v>
-      </c>
-      <c r="G3" s="4">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="3">
-        <v>61</v>
-      </c>
-      <c r="C4" s="3">
-        <v>13</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="4">
-        <v>48</v>
-      </c>
-      <c r="G4" s="4">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="3">
-        <v>62</v>
-      </c>
-      <c r="C5" s="3">
-        <v>14</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="4">
-        <v>48</v>
-      </c>
-      <c r="G5" s="4">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="3">
-        <v>60</v>
-      </c>
-      <c r="C6" s="3">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" s="4">
-        <v>46</v>
-      </c>
-      <c r="G6" s="4">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="3">
-        <v>61</v>
-      </c>
-      <c r="C7" s="3">
-        <v>14</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="4">
-        <v>48</v>
-      </c>
-      <c r="G7" s="4">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="3">
-        <v>59</v>
-      </c>
-      <c r="C8" s="3">
-        <v>13</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="4">
-        <v>46</v>
-      </c>
-      <c r="G8" s="4">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A9" s="1"/>
+    <row r="9" spans="1:6" ht="21" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C14"/>
+      <c r="D14"/>
+      <c r="E14"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C15"/>
+      <c r="D15"/>
+      <c r="E15"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+    </row>
+    <row r="17" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17"/>
+    </row>
+    <row r="18" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+    </row>
+    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
+    </row>
+    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+    </row>
+    <row r="21" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C21"/>
+      <c r="D21"/>
+      <c r="E21"/>
+    </row>
+    <row r="22" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C22"/>
+      <c r="D22"/>
+      <c r="E22"/>
+    </row>
+    <row r="23" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Revert "Removed medians and did some minor locale adjustments."
This reverts commit a04c27dc51fbc6eb29b9476872a0f6812ea31e0d.
</commit_message>
<xml_diff>
--- a/data/ref_pop-2026-03-20.xlsx
+++ b/data/ref_pop-2026-03-20.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hakanjo\ProtonDrive\My files\forskningssektionen\projects-current\jeanette_melin-shiny\share\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hakanjo\ProtonDrive\My files\forskningssektionen\projects-current\jeanette_melin-shiny\elderly_wellbeing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DB6ABB-8CB4-4B30-8BA9-AFD70C1A272C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9CD940-D41C-43C4-9EBC-07E02A37CB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11835" xr2:uid="{37809B56-4A83-7B42-93FB-B3F3B8C0AE69}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{37809B56-4A83-7B42-93FB-B3F3B8C0AE69}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
   <si>
     <t>Medelvärde</t>
   </si>
@@ -50,56 +50,59 @@
     <t>2/3 range</t>
   </si>
   <si>
-    <t>Totalt</t>
-  </si>
-  <si>
     <t> 62</t>
   </si>
   <si>
     <t>  48-73 </t>
   </si>
   <si>
-    <t>Män</t>
-  </si>
-  <si>
     <t> 60</t>
   </si>
   <si>
     <t> 46-73</t>
   </si>
   <si>
-    <t>Kvinnor</t>
-  </si>
-  <si>
     <t> 48-73</t>
   </si>
   <si>
-    <t>79 år och yngre</t>
-  </si>
-  <si>
     <t> 48-76</t>
   </si>
   <si>
-    <t>80 år och äldre</t>
-  </si>
-  <si>
-    <t>Född i Sverige</t>
-  </si>
-  <si>
-    <t>Född utanför Sverige</t>
-  </si>
-  <si>
     <t> 46-71</t>
   </si>
   <si>
-    <t>N</t>
+    <t>q_1_6</t>
+  </si>
+  <si>
+    <t>q_5_6</t>
+  </si>
+  <si>
+    <t>Totalt (ref.)</t>
+  </si>
+  <si>
+    <t>Män (ref.)</t>
+  </si>
+  <si>
+    <t>Kvinnor (ref.)</t>
+  </si>
+  <si>
+    <t>79 år och yngre (ref.)</t>
+  </si>
+  <si>
+    <t>80 år och äldre (ref.)</t>
+  </si>
+  <si>
+    <t>Född i Sverige (ref.)</t>
+  </si>
+  <si>
+    <t>Född utanför Sverige (ref.)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -125,17 +128,6 @@
       <name val="Calibri Light"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -145,7 +137,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -153,47 +145,20 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -528,234 +493,197 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F638BF61-FA25-0549-BAC0-EA20ABD1A0F5}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="10.875" style="3"/>
+    <col min="1" max="1" width="18.125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="10.875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="3">
+        <v>60</v>
+      </c>
+      <c r="C2" s="3">
+        <v>14</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="4">
+        <v>48</v>
+      </c>
+      <c r="G2" s="3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="3">
+        <v>59</v>
+      </c>
+      <c r="C3" s="3">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="4">
+        <v>46</v>
+      </c>
+      <c r="G3" s="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3">
+        <v>61</v>
+      </c>
+      <c r="C4" s="3">
+        <v>13</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="4">
+        <v>48</v>
+      </c>
+      <c r="G4" s="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3">
+        <v>62</v>
+      </c>
+      <c r="C5" s="3">
+        <v>14</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="4">
+        <v>48</v>
+      </c>
+      <c r="G5" s="4">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3">
+        <v>60</v>
+      </c>
+      <c r="C6" s="3">
+        <v>13</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4">
+        <v>46</v>
+      </c>
+      <c r="G6" s="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="B7" s="3">
+        <v>61</v>
+      </c>
+      <c r="C7" s="3">
+        <v>14</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4">
-        <v>60</v>
-      </c>
-      <c r="C2" s="4">
-        <v>14</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="4">
+        <v>48</v>
+      </c>
+      <c r="G7" s="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="3">
+        <v>59</v>
+      </c>
+      <c r="C8" s="3">
+        <v>13</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="5">
-        <v>1187</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="4">
-        <v>59</v>
-      </c>
-      <c r="C3" s="4">
-        <v>14</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="5">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="E8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="4">
-        <v>61</v>
-      </c>
-      <c r="C4" s="4">
-        <v>13</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="5">
-        <v>824</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="4">
-        <v>62</v>
-      </c>
-      <c r="C5" s="4">
-        <v>14</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="5">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="4">
-        <v>60</v>
-      </c>
-      <c r="C6" s="4">
-        <v>13</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="5">
-        <v>716</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="4">
-        <v>61</v>
-      </c>
-      <c r="C7" s="4">
-        <v>14</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="5">
-        <v>1107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="4">
-        <v>59</v>
-      </c>
-      <c r="C8" s="4">
-        <v>13</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="6">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A9" s="2"/>
-      <c r="F9" s="7"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C12"/>
-      <c r="D12"/>
-      <c r="E12"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C13"/>
-      <c r="D13"/>
-      <c r="E13"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C14"/>
-      <c r="D14"/>
-      <c r="E14"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C15"/>
-      <c r="D15"/>
-      <c r="E15"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C16"/>
-      <c r="D16"/>
-      <c r="E16"/>
-    </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C17"/>
-      <c r="D17"/>
-      <c r="E17"/>
-    </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C18"/>
-      <c r="D18"/>
-      <c r="E18"/>
-    </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C19"/>
-      <c r="D19"/>
-      <c r="E19"/>
-    </row>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C20"/>
-      <c r="D20"/>
-      <c r="E20"/>
-    </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-    </row>
-    <row r="22" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-    </row>
-    <row r="23" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C23"/>
-      <c r="D23"/>
-      <c r="E23"/>
+      <c r="F8" s="4">
+        <v>46</v>
+      </c>
+      <c r="G8" s="4">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A9" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Clarified some help messages and changed the upload template.
</commit_message>
<xml_diff>
--- a/data/ref_pop-2026-03-20.xlsx
+++ b/data/ref_pop-2026-03-20.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hakanjo\ProtonDrive\My files\forskningssektionen\projects-current\jeanette_melin-shiny\elderly_wellbeing\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9CD940-D41C-43C4-9EBC-07E02A37CB4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CBB1C20-09CE-4652-B814-A9D3A1947EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{37809B56-4A83-7B42-93FB-B3F3B8C0AE69}"/>
+    <workbookView xWindow="2790" yWindow="5115" windowWidth="21600" windowHeight="11835" xr2:uid="{37809B56-4A83-7B42-93FB-B3F3B8C0AE69}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
   <si>
     <t>Medelvärde</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>Född utanför Sverige (ref.)</t>
+  </si>
+  <si>
+    <t>n</t>
   </si>
 </sst>
 </file>
@@ -493,14 +496,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F638BF61-FA25-0549-BAC0-EA20ABD1A0F5}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="5" width="10.875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3"/>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -520,8 +523,11 @@
       <c r="G1" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
@@ -543,8 +549,11 @@
       <c r="G2" s="3">
         <v>73</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="3">
+        <v>1187</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
@@ -566,8 +575,11 @@
       <c r="G3" s="4">
         <v>73</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="3">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -589,8 +601,11 @@
       <c r="G4" s="4">
         <v>73</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" s="3">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
@@ -612,8 +627,11 @@
       <c r="G5" s="4">
         <v>76</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="3">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>17</v>
       </c>
@@ -635,8 +653,11 @@
       <c r="G6" s="4">
         <v>73</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" s="3">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
@@ -658,8 +679,11 @@
       <c r="G7" s="4">
         <v>73</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" s="3">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>19</v>
       </c>
@@ -681,8 +705,11 @@
       <c r="G8" s="4">
         <v>71</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="H8" s="3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="21" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
     </row>
   </sheetData>

</xml_diff>